<commit_message>
#5 sensors add in BOM peripherals
</commit_message>
<xml_diff>
--- a/Design Files/LogNController/BOM/eSpark BOM.xlsx
+++ b/Design Files/LogNController/BOM/eSpark BOM.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="566" uniqueCount="370">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="564" uniqueCount="369">
   <si>
     <t>Component list</t>
   </si>
@@ -1086,18 +1086,6 @@
     <t>PH Sensor</t>
   </si>
   <si>
-    <t xml:space="preserve">DS380 </t>
-  </si>
-  <si>
-    <t>Disen</t>
-  </si>
-  <si>
-    <t>Supplier Quote Required</t>
-  </si>
-  <si>
-    <t>Digital pH Sensor</t>
-  </si>
-  <si>
     <t>DC Pump</t>
   </si>
   <si>
@@ -1129,6 +1117,15 @@
   </si>
   <si>
     <t>Chipsmall</t>
+  </si>
+  <si>
+    <t>Industrial Optical DO Meter Dissolved Oxygen Sensor in Water</t>
+  </si>
+  <si>
+    <t>Alibaba</t>
+  </si>
+  <si>
+    <t>Industrial RS485 Online Water ORP PH Sensor</t>
   </si>
 </sst>
 </file>
@@ -4918,7 +4915,7 @@
       </c>
       <c r="Q65" s="13"/>
     </row>
-    <row r="66" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:17" ht="36" x14ac:dyDescent="0.25">
       <c r="A66" s="1"/>
       <c r="B66" s="16">
         <f t="shared" si="0"/>
@@ -4937,7 +4934,7 @@
         <v>332</v>
       </c>
       <c r="G66" s="13" t="s">
-        <v>355</v>
+        <v>366</v>
       </c>
       <c r="H66" s="13" t="s">
         <v>332</v>
@@ -4958,18 +4955,18 @@
         <v>1</v>
       </c>
       <c r="N66" s="46" t="s">
-        <v>356</v>
-      </c>
-      <c r="O66" s="14"/>
+        <v>367</v>
+      </c>
+      <c r="O66" s="14">
+        <v>125.8</v>
+      </c>
       <c r="P66" s="14">
         <f t="shared" si="28"/>
-        <v>0</v>
-      </c>
-      <c r="Q66" s="47" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="67" spans="1:17" x14ac:dyDescent="0.25">
+        <v>125.8</v>
+      </c>
+      <c r="Q66" s="47"/>
+    </row>
+    <row r="67" spans="1:17" ht="24" x14ac:dyDescent="0.25">
       <c r="A67" s="1"/>
       <c r="B67" s="16">
         <f t="shared" si="0"/>
@@ -4988,7 +4985,7 @@
         <v>332</v>
       </c>
       <c r="G67" s="13" t="s">
-        <v>358</v>
+        <v>368</v>
       </c>
       <c r="H67" s="13" t="s">
         <v>332</v>
@@ -5009,16 +5006,16 @@
         <v>1</v>
       </c>
       <c r="N67" s="46" t="s">
-        <v>356</v>
-      </c>
-      <c r="O67" s="14"/>
+        <v>367</v>
+      </c>
+      <c r="O67" s="14">
+        <v>62.9</v>
+      </c>
       <c r="P67" s="14">
         <f t="shared" si="28"/>
-        <v>0</v>
-      </c>
-      <c r="Q67" s="47" t="s">
-        <v>357</v>
-      </c>
+        <v>62.9</v>
+      </c>
+      <c r="Q67" s="47"/>
     </row>
     <row r="68" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A68" s="1"/>
@@ -5030,19 +5027,19 @@
         <v>340</v>
       </c>
       <c r="D68" s="13" t="s">
-        <v>359</v>
+        <v>355</v>
       </c>
       <c r="E68" s="13" t="s">
-        <v>366</v>
+        <v>362</v>
       </c>
       <c r="F68" s="13" t="s">
         <v>332</v>
       </c>
       <c r="G68" s="13" t="s">
-        <v>365</v>
+        <v>361</v>
       </c>
       <c r="H68" s="13" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="I68" s="13" t="s">
         <v>332</v>
@@ -5070,7 +5067,7 @@
         <v>90.99</v>
       </c>
       <c r="Q68" s="47" t="s">
-        <v>368</v>
+        <v>364</v>
       </c>
     </row>
     <row r="69" spans="1:17" x14ac:dyDescent="0.25">
@@ -5083,19 +5080,19 @@
         <v>340</v>
       </c>
       <c r="D69" s="13" t="s">
-        <v>360</v>
+        <v>356</v>
       </c>
       <c r="E69" s="13" t="s">
-        <v>363</v>
+        <v>359</v>
       </c>
       <c r="F69" s="13" t="s">
         <v>332</v>
       </c>
       <c r="G69" s="13" t="s">
-        <v>361</v>
+        <v>357</v>
       </c>
       <c r="H69" s="13" t="s">
-        <v>364</v>
+        <v>360</v>
       </c>
       <c r="I69" s="13" t="s">
         <v>332</v>
@@ -5134,7 +5131,7 @@
         <v>340</v>
       </c>
       <c r="D70" s="13" t="s">
-        <v>362</v>
+        <v>358</v>
       </c>
       <c r="E70" s="13"/>
       <c r="F70" s="13"/>
@@ -5193,7 +5190,7 @@
         <v>1</v>
       </c>
       <c r="N71" s="46" t="s">
-        <v>369</v>
+        <v>365</v>
       </c>
       <c r="O71" s="14">
         <v>60.87</v>
@@ -5224,7 +5221,7 @@
       <c r="O72" s="50"/>
       <c r="P72" s="17">
         <f>SUM(P8:P71)</f>
-        <v>251.96009999999998</v>
+        <v>440.6601</v>
       </c>
       <c r="Q72" s="1"/>
     </row>
@@ -5314,11 +5311,11 @@
     <hyperlink ref="N63" r:id="rId56"/>
     <hyperlink ref="N64" r:id="rId57"/>
     <hyperlink ref="N65" r:id="rId58"/>
-    <hyperlink ref="N66" r:id="rId59"/>
-    <hyperlink ref="N67" r:id="rId60"/>
-    <hyperlink ref="N69" r:id="rId61"/>
-    <hyperlink ref="N68" r:id="rId62"/>
-    <hyperlink ref="N71" r:id="rId63"/>
+    <hyperlink ref="N69" r:id="rId59"/>
+    <hyperlink ref="N68" r:id="rId60"/>
+    <hyperlink ref="N71" r:id="rId61"/>
+    <hyperlink ref="N66" r:id="rId62"/>
+    <hyperlink ref="N67" r:id="rId63"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId64"/>

</xml_diff>